<commit_message>
Added remaining Test Design and Test Case Specifications to the Test Design folder
</commit_message>
<xml_diff>
--- a/Test Design/Test Case Specifications_04.01 Create General Ledger Accounts_Thyagaraj Raghava_C1.xlsx
+++ b/Test Design/Test Case Specifications_04.01 Create General Ledger Accounts_Thyagaraj Raghava_C1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danfox/dev/Old-Documents/Pace/Fall 2025/Applied Software Testing/GitHub Repo/CS696F-Team1/Test Design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87FCA5D8-C954-2A43-8D9C-05923FDAD65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FF9A4D-388F-C74D-A2E6-739AF80FF915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17460" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4420" yWindow="680" windowWidth="25820" windowHeight="18960" firstSheet="4" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="12" r:id="rId1"/>
@@ -2037,6 +2037,55 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>523875</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>361950</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>476250</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FC11A101-7FCA-57A5-2265-DCC6615D9FC3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7896225" y="76200"/>
+          <a:ext cx="8105775" cy="3962400"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
@@ -3516,6 +3565,7 @@
     <mergeCell ref="B8:D10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>